<commit_message>
Added Inspections and checkstyle used
Moved product and sprint backlog to correct place
</commit_message>
<xml_diff>
--- a/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
+++ b/sprints/sprint1/Sprint Backlog & Burnup Chart.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29825"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/jcorley_westga_edu/Documents/Teaching/Software Engineering II/SE2 - Spring 2026/Project/SE2-project-repos-sample/sprints/sprint1/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://westga365-my.sharepoint.com/personal/kd00250_my_westga_edu/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="13_ncr:1_{9C9C4265-351C-41A0-89E5-93A08D9C51A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C68B4513-1541-415B-8F23-00764467EF2F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{ED044FEF-8882-495A-892E-3CD3C9543B0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="75">
+  <si>
+    <t>Who's Implementing</t>
+  </si>
   <si>
     <t>Related User Story</t>
   </si>
@@ -47,6 +50,9 @@
     <t>Initial Estimate</t>
   </si>
   <si>
+    <t>Amount Worked on…</t>
+  </si>
+  <si>
     <t>Week 1</t>
   </si>
   <si>
@@ -59,23 +65,209 @@
     <t>Week 4</t>
   </si>
   <si>
-    <t>Amount Remaining After…</t>
+    <t>Jake</t>
+  </si>
+  <si>
+    <t>Login</t>
+  </si>
+  <si>
+    <t>Create GUI login</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create tag </t>
+  </si>
+  <si>
+    <t>Create the code behind for the create tag page</t>
+  </si>
+  <si>
+    <t>Update GUI to work with updated design</t>
+  </si>
+  <si>
+    <t>Update Codebehind to work with updated GUI</t>
+  </si>
+  <si>
+    <t>Update View model to work with updated codebehind</t>
+  </si>
+  <si>
+    <t>Update business logic to add tags to projects</t>
+  </si>
+  <si>
+    <t>Update testing in create tags</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jake </t>
+  </si>
+  <si>
+    <t>Bind the codebehind to the gui (view) for the create tag page</t>
+  </si>
+  <si>
+    <t>Create business functionality for create tags</t>
+  </si>
+  <si>
+    <t>Test create tags business logic</t>
+  </si>
+  <si>
+    <t>Update test cases to test updated create tag logic</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Connect GUI to work with other pages </t>
+  </si>
+  <si>
+    <t>Jake, Matthew, Kenny, Mark</t>
+  </si>
+  <si>
+    <t>Animal Tracking System</t>
+  </si>
+  <si>
+    <t>Meeting 1</t>
+  </si>
+  <si>
+    <t>Meeting 2</t>
+  </si>
+  <si>
+    <t>Meeting 3</t>
+  </si>
+  <si>
+    <t>Kenneth</t>
+  </si>
+  <si>
+    <t>Create tag / Login / Create Project</t>
+  </si>
+  <si>
+    <t>Created the data storage class that acted as our data base for the mock server</t>
+  </si>
+  <si>
+    <t>Add User</t>
+  </si>
+  <si>
+    <t>Create the business functionality for adding a user to the system</t>
+  </si>
+  <si>
+    <t>Create the Gui for adding a user</t>
+  </si>
+  <si>
+    <t>Create the codebehind for the add user page</t>
+  </si>
+  <si>
+    <t>Bind the codebehind to the gui (view) for the add user page</t>
+  </si>
+  <si>
+    <t>Create Project</t>
+  </si>
+  <si>
+    <t>Bind the gui to the codebehind (view) for the create project page</t>
+  </si>
+  <si>
+    <t>Add/Remove Scientist</t>
+  </si>
+  <si>
+    <t>Create business functionality for adding and removing a scientist to/from a project</t>
+  </si>
+  <si>
+    <t>Modify to the codebehind as necessary (functionality could be coupled to admin main page)</t>
+  </si>
+  <si>
+    <t>View Project Data</t>
+  </si>
+  <si>
+    <t>Create the business logic for viewing project data</t>
+  </si>
+  <si>
+    <t>Create the gui for displaying the project data</t>
+  </si>
+  <si>
+    <t>Create the codebehind for the view project data page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">view project data </t>
+  </si>
+  <si>
+    <t>Bind the viewmodel to the gui (view) for the view project data page</t>
+  </si>
+  <si>
+    <t>Kenneth/Matthew</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fixed .idea being tracked and cleaned up project </t>
+  </si>
+  <si>
+    <t>design descussion</t>
+  </si>
+  <si>
+    <t>Mark</t>
+  </si>
+  <si>
+    <t>Create gui for the create project page</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create Project </t>
+  </si>
+  <si>
+    <t>Create the business logic for creating a project</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delete Project </t>
+  </si>
+  <si>
+    <t>Create Gui for the delete project page</t>
+  </si>
+  <si>
+    <t>Create Business functionality for deleting a project</t>
+  </si>
+  <si>
+    <t>Create the codebehind for the delete project page</t>
+  </si>
+  <si>
+    <t>bind the codebehind to the gui (view) for the delete project page</t>
+  </si>
+  <si>
+    <t>Mark/Kenneth</t>
+  </si>
+  <si>
+    <t>Create the code behind for the create project page</t>
+  </si>
+  <si>
+    <t>Matthew</t>
+  </si>
+  <si>
+    <t>Login (Admin)</t>
+  </si>
+  <si>
+    <t>create the admin user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create the gui for the start up page </t>
+  </si>
+  <si>
+    <t>Bind the gui to the codebehind (view) for the login page</t>
+  </si>
+  <si>
+    <t>Create business logic for login</t>
+  </si>
+  <si>
+    <t>Create model implementation for gui</t>
+  </si>
+  <si>
+    <t>Create the gui for the create tag page</t>
+  </si>
+  <si>
+    <t>Create storage and local server for data</t>
   </si>
   <si>
     <t>Estimate Totals</t>
   </si>
   <si>
-    <t>Code Things…</t>
-  </si>
-  <si>
-    <t>That User Story</t>
+    <t>Estimation Totals</t>
+  </si>
+  <si>
+    <t>Total sums</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -92,7 +284,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -129,6 +321,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -142,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
@@ -151,11 +349,15 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -252,6 +454,9 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:tx>
+            <c:v>Estimated Total Hours</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -266,21 +471,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$27:$G$27</c:f>
+              <c:f>Sheet1!$E$46:$H$46</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>25</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>50</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>75</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -288,13 +493,16 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-48A7-4DCE-854F-20166BFB91ED}"/>
+              <c16:uniqueId val="{00000000-3DA4-4256-AC6D-A806AD4E2E5F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
           <c:idx val="1"/>
           <c:order val="1"/>
+          <c:tx>
+            <c:v>Hours Worked On</c:v>
+          </c:tx>
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
@@ -309,21 +517,21 @@
           </c:marker>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$28:$G$28</c:f>
+              <c:f>Sheet1!$E$47:$H$47</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
-                  <c:v>100</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>100</c:v>
+                  <c:v>42</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>100</c:v>
+                  <c:v>73</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>100</c:v>
+                  <c:v>101</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -331,7 +539,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-48A7-4DCE-854F-20166BFB91ED}"/>
+              <c16:uniqueId val="{00000002-3DA4-4256-AC6D-A806AD4E2E5F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -344,11 +552,11 @@
           <c:showBubbleSize val="0"/>
         </c:dLbls>
         <c:smooth val="0"/>
-        <c:axId val="2056245824"/>
-        <c:axId val="2056242944"/>
+        <c:axId val="1121534472"/>
+        <c:axId val="1121537032"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2056245824"/>
+        <c:axId val="1121534472"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -390,7 +598,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2056242944"/>
+        <c:crossAx val="1121537032"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -398,7 +606,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="2056242944"/>
+        <c:axId val="1121537032"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -449,7 +657,7 @@
             <a:endParaRPr lang="en-US"/>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2056245824"/>
+        <c:crossAx val="1121534472"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -461,16 +669,40 @@
         <a:effectLst/>
       </c:spPr>
     </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1">
+                  <a:lumMod val="65000"/>
+                  <a:lumOff val="35000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:defRPr>
+          </a:pPr>
+          <a:endParaRPr lang="en-US"/>
+        </a:p>
+      </c:txPr>
+    </c:legend>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
     <c:showDLblsOverMax val="0"/>
-    <c:extLst>
-      <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
-        <c16r3:dataDisplayOptions16>
-          <c16r3:dispNaAsBlank val="1"/>
-        </c16r3:dataDisplayOptions16>
-      </c:ext>
-    </c:extLst>
   </c:chart>
   <c:spPr>
     <a:solidFill>
@@ -1066,22 +1298,25 @@
   <xdr:twoCellAnchor>
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>38100</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>100012</xdr:rowOff>
+      <xdr:colOff>409575</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>133350</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>342900</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>176212</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
-        <xdr:cNvPr id="3" name="Chart 2">
+        <xdr:cNvPr id="7" name="Chart 6">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{64F532F7-5440-F07B-5C89-7E5BCBF73E65}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0E0C8C3-3570-C04B-D5CD-63BC1B1C7853}"/>
+            </a:ext>
+            <a:ext uri="{147F2762-F138-4A5C-976F-8EAC2B608ADB}">
+              <a16:predDERef xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" pred="{64F532F7-5440-F07B-5C89-7E5BCBF73E65}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1365,327 +1600,980 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G28"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:H47"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="51.42578125" customWidth="1"/>
-    <col min="2" max="2" width="41.7109375" customWidth="1"/>
-    <col min="3" max="3" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="51.42578125" customWidth="1"/>
+    <col min="3" max="3" width="41.7109375" customWidth="1"/>
+    <col min="4" max="4" width="15.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:8">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="7" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="6" t="s">
+      <c r="B1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
+    </row>
+    <row r="2" spans="1:8">
+      <c r="A2" s="8"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="G2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" s="7"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="5" t="s">
-        <v>3</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>4</v>
-      </c>
-      <c r="F2" s="5" t="s">
-        <v>5</v>
-      </c>
-      <c r="G2" s="5" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="H2" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8">
       <c r="A3" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2">
+        <v>1</v>
+      </c>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+    </row>
+    <row r="4" spans="1:8">
+      <c r="A4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="1">
-        <v>100</v>
-      </c>
-      <c r="D3" s="2">
-        <v>25</v>
-      </c>
-      <c r="E3" s="2">
-        <v>50</v>
-      </c>
-      <c r="F3" s="2">
-        <v>75</v>
-      </c>
-      <c r="G3" s="2">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A4" s="1"/>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="B4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" s="1">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2">
+        <v>2</v>
+      </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="2"/>
+      <c r="H4" s="2"/>
+    </row>
+    <row r="5" spans="1:8">
+      <c r="A5" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="1">
+        <v>1</v>
+      </c>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="2"/>
+      <c r="G5" s="2">
+        <v>1</v>
+      </c>
+      <c r="H5" s="2"/>
+    </row>
+    <row r="6" spans="1:8">
+      <c r="A6" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D6" s="1">
+        <v>2</v>
+      </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="1"/>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="2"/>
+      <c r="G6" s="2">
+        <v>2</v>
+      </c>
+      <c r="H6" s="2"/>
+    </row>
+    <row r="7" spans="1:8" ht="30">
+      <c r="A7" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D7" s="1">
+        <v>1</v>
+      </c>
       <c r="E7" s="2"/>
       <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="1"/>
-      <c r="B8" s="1"/>
-      <c r="C8" s="1"/>
-      <c r="D8" s="2"/>
+      <c r="G7" s="2">
+        <v>2</v>
+      </c>
+      <c r="H7" s="2"/>
+    </row>
+    <row r="8" spans="1:8">
+      <c r="A8" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="1">
+        <v>1</v>
+      </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="1"/>
-      <c r="B9" s="1"/>
-      <c r="C9" s="1"/>
-      <c r="D9" s="2"/>
+      <c r="H8" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8">
+      <c r="A9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="1">
+        <v>1</v>
+      </c>
       <c r="E9" s="2"/>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="1"/>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
+      <c r="H9" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30">
+      <c r="A10" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
       <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
+      <c r="F10" s="2">
+        <v>1</v>
+      </c>
       <c r="G10" s="2"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="1"/>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
+      <c r="H10" s="2"/>
+    </row>
+    <row r="11" spans="1:8">
+      <c r="A11" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2</v>
+      </c>
       <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+      <c r="F11" s="2">
+        <v>4</v>
+      </c>
       <c r="G11" s="2"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="1"/>
-      <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="H11" s="2"/>
+    </row>
+    <row r="12" spans="1:8">
+      <c r="A12" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="1">
+        <v>2</v>
+      </c>
+      <c r="E12" s="2">
+        <v>3</v>
+      </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="1"/>
-      <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="1:8" ht="30">
+      <c r="A13" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="D13" s="1">
+        <v>1</v>
+      </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="1"/>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
+      <c r="G13" s="2">
+        <v>1</v>
+      </c>
+      <c r="H13" s="2"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D14" s="1">
+        <v>2</v>
+      </c>
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
       <c r="G14" s="2"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="1"/>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="H14" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8">
+      <c r="A15" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D15" s="1">
+        <v>2</v>
+      </c>
+      <c r="E15" s="2">
+        <v>2</v>
+      </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="1"/>
-      <c r="B16" s="1"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="1:8">
+      <c r="A16" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D16" s="1">
+        <v>3</v>
+      </c>
       <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="F16" s="2">
+        <v>3</v>
+      </c>
       <c r="G16" s="2"/>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="1"/>
-      <c r="B17" s="1"/>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
+      <c r="H16" s="2"/>
+    </row>
+    <row r="17" spans="1:8">
+      <c r="A17" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="1">
+        <v>5</v>
+      </c>
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A18" s="1"/>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
+      <c r="H17" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" ht="30.75">
+      <c r="A18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D18" s="1">
+        <v>3</v>
+      </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="1"/>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="2"/>
+      <c r="G18" s="2">
+        <v>4</v>
+      </c>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" ht="29.25" customHeight="1">
+      <c r="A19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="1">
+        <v>4</v>
+      </c>
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="1"/>
-      <c r="B20" s="1"/>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
+      <c r="G19" s="2">
+        <v>5</v>
+      </c>
+      <c r="H19" s="2"/>
+    </row>
+    <row r="20" spans="1:8">
+      <c r="A20" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="D20" s="1">
+        <v>1</v>
+      </c>
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="1"/>
-      <c r="B21" s="1"/>
-      <c r="C21" s="1"/>
-      <c r="D21" s="2"/>
+      <c r="H20" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D21" s="1">
+        <v>1</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A22" s="1"/>
-      <c r="B22" s="1"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
+      <c r="G21" s="2">
+        <v>1</v>
+      </c>
+      <c r="H21" s="2"/>
+    </row>
+    <row r="22" spans="1:8" ht="30">
+      <c r="A22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="1">
+        <v>2</v>
+      </c>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="1"/>
-      <c r="B23" s="1"/>
-      <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
+      <c r="H22" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" ht="30">
+      <c r="A23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="D23" s="1">
+        <v>3</v>
+      </c>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
+      <c r="H23" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" ht="30">
+      <c r="A24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D24" s="1">
+        <v>2</v>
+      </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
-    </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
+      <c r="H24" s="2">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" ht="45">
+      <c r="A25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="D25" s="1">
+        <v>1</v>
+      </c>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
-    </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="2"/>
+      <c r="H25" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" ht="30">
+      <c r="A26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="1">
+        <v>1</v>
+      </c>
       <c r="E26" s="2"/>
-      <c r="F26" s="2"/>
+      <c r="F26" s="2">
+        <v>3</v>
+      </c>
       <c r="G26" s="2"/>
-    </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="B27" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C27" s="3">
-        <f>SUM(C3:C26)</f>
-        <v>100</v>
-      </c>
-      <c r="D27" s="3">
-        <f t="shared" ref="D27:G27" si="0">SUM(D3:D26)</f>
-        <v>25</v>
-      </c>
-      <c r="E27" s="3">
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D27" s="1">
+        <v>1</v>
+      </c>
+      <c r="E27" s="2">
+        <v>3</v>
+      </c>
+      <c r="F27" s="2"/>
+      <c r="G27" s="2"/>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" ht="30">
+      <c r="A28" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="C28" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D28" s="1">
+        <v>3</v>
+      </c>
+      <c r="E28" s="2">
+        <v>2</v>
+      </c>
+      <c r="F28" s="2">
+        <v>1</v>
+      </c>
+      <c r="G28" s="2"/>
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="1:8" ht="30">
+      <c r="A29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="D29" s="1">
+        <v>2</v>
+      </c>
+      <c r="E29" s="2"/>
+      <c r="F29" s="2"/>
+      <c r="G29" s="2"/>
+      <c r="H29" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8">
+      <c r="A30" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D30" s="1">
+        <v>1</v>
+      </c>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2">
+        <v>2</v>
+      </c>
+      <c r="G30" s="2"/>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="1"/>
+      <c r="E31" s="2">
+        <v>1</v>
+      </c>
+      <c r="F31" s="2">
+        <v>1</v>
+      </c>
+      <c r="G31" s="2"/>
+      <c r="H31" s="2"/>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" s="1">
+        <v>2</v>
+      </c>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2">
+        <v>2</v>
+      </c>
+      <c r="G32" s="2">
+        <v>2</v>
+      </c>
+      <c r="H32" s="2"/>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C33" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="D33" s="1">
+        <v>1</v>
+      </c>
+      <c r="E33" s="2">
+        <v>1</v>
+      </c>
+      <c r="F33" s="2"/>
+      <c r="G33" s="2"/>
+      <c r="H33" s="2"/>
+    </row>
+    <row r="34" spans="1:8" ht="30">
+      <c r="A34" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C34" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="1">
+        <v>3</v>
+      </c>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2">
+        <v>2</v>
+      </c>
+      <c r="G34" s="2">
+        <v>3</v>
+      </c>
+      <c r="H34" s="2"/>
+    </row>
+    <row r="35" spans="1:8" ht="30">
+      <c r="A35" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C35" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D35" s="1">
+        <v>2</v>
+      </c>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2">
+        <v>2</v>
+      </c>
+      <c r="H35" s="2"/>
+    </row>
+    <row r="36" spans="1:8" ht="30">
+      <c r="A36" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="C36" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="D36" s="1">
+        <v>1</v>
+      </c>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2">
+        <v>1</v>
+      </c>
+      <c r="H36" s="2"/>
+    </row>
+    <row r="37" spans="1:8" ht="30">
+      <c r="A37" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>62</v>
+      </c>
+      <c r="D37" s="1">
+        <v>2</v>
+      </c>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2">
+        <v>1</v>
+      </c>
+      <c r="G37" s="2"/>
+      <c r="H37" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="D38" s="1">
+        <v>1</v>
+      </c>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2">
+        <v>1</v>
+      </c>
+      <c r="H38" s="2"/>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C39" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D39" s="1">
+        <v>1</v>
+      </c>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2">
+        <v>2</v>
+      </c>
+      <c r="G39" s="2"/>
+      <c r="H39" s="2"/>
+    </row>
+    <row r="40" spans="1:8" ht="30">
+      <c r="A40" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C40" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D40" s="1">
+        <v>1</v>
+      </c>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2">
+        <v>2</v>
+      </c>
+      <c r="G40" s="2"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="1:8">
+      <c r="A41" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C41" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="D41" s="1">
+        <v>2</v>
+      </c>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+      <c r="G41" s="2">
+        <v>3</v>
+      </c>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="1:8">
+      <c r="A42" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D42" s="1">
+        <v>1</v>
+      </c>
+      <c r="E42" s="2">
+        <v>1</v>
+      </c>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" spans="1:8">
+      <c r="A43" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D43" s="1">
+        <v>1</v>
+      </c>
+      <c r="E43" s="2">
+        <v>2</v>
+      </c>
+      <c r="F43" s="2"/>
+      <c r="G43" s="2"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D44" s="1">
+        <v>4</v>
+      </c>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+      <c r="G44" s="2">
+        <v>3</v>
+      </c>
+      <c r="H44" s="2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="C45" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D45" s="3">
+        <f>SUM(D3:D44)</f>
+        <v>73</v>
+      </c>
+      <c r="E45" s="3">
+        <f>SUM(E3:E44)</f>
+        <v>18</v>
+      </c>
+      <c r="F45" s="3">
+        <f>SUM(F3:F44)</f>
+        <v>24</v>
+      </c>
+      <c r="G45" s="3">
+        <f>SUM(G3:G44)</f>
+        <v>31</v>
+      </c>
+      <c r="H45" s="3">
+        <f>SUM(H3:H44)</f>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="D46" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="E46" s="3">
+        <f>$D$45</f>
+        <v>73</v>
+      </c>
+      <c r="F46" s="3">
+        <f t="shared" ref="F46:H46" si="0">$D$45</f>
+        <v>73</v>
+      </c>
+      <c r="G46" s="3">
         <f t="shared" si="0"/>
-        <v>50</v>
-      </c>
-      <c r="F27" s="3">
+        <v>73</v>
+      </c>
+      <c r="H46" s="3">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="G27" s="3">
-        <f t="shared" si="0"/>
-        <v>100</v>
-      </c>
-    </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="D28">
-        <f>$C$27</f>
-        <v>100</v>
-      </c>
-      <c r="E28">
-        <f t="shared" ref="E28:G28" si="1">$C$27</f>
-        <v>100</v>
-      </c>
-      <c r="F28">
-        <f t="shared" si="1"/>
-        <v>100</v>
-      </c>
-      <c r="G28">
-        <f t="shared" si="1"/>
-        <v>100</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="D47" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E47" s="3">
+        <f>E45</f>
+        <v>18</v>
+      </c>
+      <c r="F47" s="3">
+        <f>F45+E47</f>
+        <v>42</v>
+      </c>
+      <c r="G47" s="3">
+        <f>G45+F47</f>
+        <v>73</v>
+      </c>
+      <c r="H47" s="3">
+        <f>H45+G47</f>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="D1:G1"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A3:H44">
+    <sortCondition ref="A3:A44"/>
+  </sortState>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="E1:H1"/>
+    <mergeCell ref="D1:D2"/>
     <mergeCell ref="C1:C2"/>
     <mergeCell ref="B1:B2"/>
-    <mergeCell ref="A1:A2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>